<commit_message>
Fix terminology of yield components i.e., Spike = Chaff + Grain
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/WaggaWagga2024/WaggaWagga2024.xlsx
+++ b/Tests/Validation/Wheat/WaggaWagga2024/WaggaWagga2024.xlsx
@@ -20027,7 +20027,7 @@
       <c r="F722"/>
       <c r="G722"/>
       <c r="H722" t="n">
-        <v>258.581420636984</v>
+        <v>902.94250132251</v>
       </c>
       <c r="I722"/>
       <c r="J722"/>
@@ -20054,7 +20054,7 @@
       <c r="F723"/>
       <c r="G723"/>
       <c r="H723" t="n">
-        <v>271.553119160093</v>
+        <v>916.838411537101</v>
       </c>
       <c r="I723"/>
       <c r="J723"/>
@@ -20081,7 +20081,7 @@
       <c r="F724"/>
       <c r="G724"/>
       <c r="H724" t="n">
-        <v>283.244195865873</v>
+        <v>996.270434332054</v>
       </c>
       <c r="I724"/>
       <c r="J724"/>
@@ -20108,7 +20108,7 @@
       <c r="F725"/>
       <c r="G725"/>
       <c r="H725" t="n">
-        <v>270.1648172525</v>
+        <v>924.207952117844</v>
       </c>
       <c r="I725"/>
       <c r="J725"/>
@@ -20135,7 +20135,7 @@
       <c r="F726"/>
       <c r="G726"/>
       <c r="H726" t="n">
-        <v>264.548506655481</v>
+        <v>877.737898261038</v>
       </c>
       <c r="I726"/>
       <c r="J726"/>
@@ -20162,7 +20162,7 @@
       <c r="F727"/>
       <c r="G727"/>
       <c r="H727" t="n">
-        <v>257.402949208964</v>
+        <v>900.524216280997</v>
       </c>
       <c r="I727"/>
       <c r="J727"/>
@@ -20189,7 +20189,7 @@
       <c r="F728"/>
       <c r="G728"/>
       <c r="H728" t="n">
-        <v>230.222750520773</v>
+        <v>810.184503919533</v>
       </c>
       <c r="I728"/>
       <c r="J728"/>
@@ -20216,7 +20216,7 @@
       <c r="F729"/>
       <c r="G729"/>
       <c r="H729" t="n">
-        <v>265.186988921777</v>
+        <v>1009.06459915201</v>
       </c>
       <c r="I729"/>
       <c r="J729"/>
@@ -20243,7 +20243,7 @@
       <c r="F730"/>
       <c r="G730"/>
       <c r="H730" t="n">
-        <v>274.17361739936</v>
+        <v>849.989592528135</v>
       </c>
       <c r="I730"/>
       <c r="J730"/>
@@ -20270,7 +20270,7 @@
       <c r="F731"/>
       <c r="G731"/>
       <c r="H731" t="n">
-        <v>282.688648589262</v>
+        <v>950.255120938897</v>
       </c>
       <c r="I731"/>
       <c r="J731"/>
@@ -20297,7 +20297,7 @@
       <c r="F732"/>
       <c r="G732"/>
       <c r="H732" t="n">
-        <v>269.910861566965</v>
+        <v>945.021012590105</v>
       </c>
       <c r="I732"/>
       <c r="J732"/>
@@ -20324,7 +20324,7 @@
       <c r="F733"/>
       <c r="G733"/>
       <c r="H733" t="n">
-        <v>251.607810105658</v>
+        <v>926.208593773007</v>
       </c>
       <c r="I733"/>
       <c r="J733"/>
@@ -20351,7 +20351,7 @@
       <c r="F734"/>
       <c r="G734"/>
       <c r="H734" t="n">
-        <v>336.236053339716</v>
+        <v>1045.19222271131</v>
       </c>
       <c r="I734"/>
       <c r="J734"/>
@@ -20378,7 +20378,7 @@
       <c r="F735"/>
       <c r="G735"/>
       <c r="H735" t="n">
-        <v>245.542051418169</v>
+        <v>834.101160611674</v>
       </c>
       <c r="I735"/>
       <c r="J735"/>
@@ -20405,7 +20405,7 @@
       <c r="F736"/>
       <c r="G736"/>
       <c r="H736" t="n">
-        <v>294.871379752884</v>
+        <v>1025.89194468028</v>
       </c>
       <c r="I736"/>
       <c r="J736"/>
@@ -20432,7 +20432,7 @@
       <c r="F737"/>
       <c r="G737"/>
       <c r="H737" t="n">
-        <v>235.121968352509</v>
+        <v>816.865684558279</v>
       </c>
       <c r="I737"/>
       <c r="J737"/>
@@ -23046,7 +23046,7 @@
       <c r="I834"/>
       <c r="J834"/>
       <c r="K834" t="n">
-        <v>902.94250132251</v>
+        <v>258.581420636984</v>
       </c>
       <c r="L834"/>
       <c r="M834"/>
@@ -23073,7 +23073,7 @@
       <c r="I835"/>
       <c r="J835"/>
       <c r="K835" t="n">
-        <v>916.838411537101</v>
+        <v>271.553119160093</v>
       </c>
       <c r="L835"/>
       <c r="M835"/>
@@ -23100,7 +23100,7 @@
       <c r="I836"/>
       <c r="J836"/>
       <c r="K836" t="n">
-        <v>996.270434332054</v>
+        <v>283.244195865873</v>
       </c>
       <c r="L836"/>
       <c r="M836"/>
@@ -23127,7 +23127,7 @@
       <c r="I837"/>
       <c r="J837"/>
       <c r="K837" t="n">
-        <v>924.207952117844</v>
+        <v>270.1648172525</v>
       </c>
       <c r="L837"/>
       <c r="M837"/>
@@ -23154,7 +23154,7 @@
       <c r="I838"/>
       <c r="J838"/>
       <c r="K838" t="n">
-        <v>877.737898261038</v>
+        <v>264.548506655481</v>
       </c>
       <c r="L838"/>
       <c r="M838"/>
@@ -23181,7 +23181,7 @@
       <c r="I839"/>
       <c r="J839"/>
       <c r="K839" t="n">
-        <v>900.524216280997</v>
+        <v>257.402949208964</v>
       </c>
       <c r="L839"/>
       <c r="M839"/>
@@ -23208,7 +23208,7 @@
       <c r="I840"/>
       <c r="J840"/>
       <c r="K840" t="n">
-        <v>810.184503919533</v>
+        <v>230.222750520773</v>
       </c>
       <c r="L840"/>
       <c r="M840"/>
@@ -23235,7 +23235,7 @@
       <c r="I841"/>
       <c r="J841"/>
       <c r="K841" t="n">
-        <v>1009.06459915201</v>
+        <v>265.186988921777</v>
       </c>
       <c r="L841"/>
       <c r="M841"/>
@@ -23262,7 +23262,7 @@
       <c r="I842"/>
       <c r="J842"/>
       <c r="K842" t="n">
-        <v>849.989592528135</v>
+        <v>274.17361739936</v>
       </c>
       <c r="L842"/>
       <c r="M842"/>
@@ -23289,7 +23289,7 @@
       <c r="I843"/>
       <c r="J843"/>
       <c r="K843" t="n">
-        <v>950.255120938897</v>
+        <v>282.688648589262</v>
       </c>
       <c r="L843"/>
       <c r="M843"/>
@@ -23316,7 +23316,7 @@
       <c r="I844"/>
       <c r="J844"/>
       <c r="K844" t="n">
-        <v>945.021012590105</v>
+        <v>269.910861566965</v>
       </c>
       <c r="L844"/>
       <c r="M844"/>
@@ -23343,7 +23343,7 @@
       <c r="I845"/>
       <c r="J845"/>
       <c r="K845" t="n">
-        <v>926.208593773007</v>
+        <v>251.607810105658</v>
       </c>
       <c r="L845"/>
       <c r="M845"/>
@@ -23370,7 +23370,7 @@
       <c r="I846"/>
       <c r="J846"/>
       <c r="K846" t="n">
-        <v>1045.19222271131</v>
+        <v>336.236053339716</v>
       </c>
       <c r="L846"/>
       <c r="M846"/>
@@ -23397,7 +23397,7 @@
       <c r="I847"/>
       <c r="J847"/>
       <c r="K847" t="n">
-        <v>834.101160611674</v>
+        <v>245.542051418169</v>
       </c>
       <c r="L847"/>
       <c r="M847"/>
@@ -23424,7 +23424,7 @@
       <c r="I848"/>
       <c r="J848"/>
       <c r="K848" t="n">
-        <v>1025.89194468028</v>
+        <v>294.871379752884</v>
       </c>
       <c r="L848"/>
       <c r="M848"/>
@@ -23451,7 +23451,7 @@
       <c r="I849"/>
       <c r="J849"/>
       <c r="K849" t="n">
-        <v>816.865684558279</v>
+        <v>235.121968352509</v>
       </c>
       <c r="L849"/>
       <c r="M849"/>

</xml_diff>